<commit_message>
20260630 commit : today, finished
</commit_message>
<xml_diff>
--- a/명세서(3조, 팀명 딱코).xlsx
+++ b/명세서(3조, 팀명 딱코).xlsx
@@ -10837,7 +10837,7 @@
       <charset val="129"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -10880,6 +10880,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -10905,7 +10911,7 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -11047,6 +11053,15 @@
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
@@ -11065,14 +11080,11 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -11399,7 +11411,7 @@
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="47" t="s">
+      <c r="B3" s="50" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="10" t="s">
@@ -11417,7 +11429,7 @@
       <c r="A4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="48"/>
+      <c r="B4" s="51"/>
       <c r="C4" s="10" t="s">
         <v>7</v>
       </c>
@@ -11433,7 +11445,7 @@
       <c r="A5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="48"/>
+      <c r="B5" s="51"/>
       <c r="C5" s="10" t="s">
         <v>7</v>
       </c>
@@ -11449,7 +11461,7 @@
       <c r="A6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="48"/>
+      <c r="B6" s="51"/>
       <c r="C6" s="10" t="s">
         <v>17</v>
       </c>
@@ -11465,7 +11477,7 @@
       <c r="A7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="48"/>
+      <c r="B7" s="51"/>
       <c r="C7" s="10" t="s">
         <v>17</v>
       </c>
@@ -11481,7 +11493,7 @@
       <c r="A8" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="48"/>
+      <c r="B8" s="51"/>
       <c r="C8" s="10" t="s">
         <v>17</v>
       </c>
@@ -11497,7 +11509,7 @@
       <c r="A9" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="48"/>
+      <c r="B9" s="51"/>
       <c r="C9" s="10" t="s">
         <v>17</v>
       </c>
@@ -11513,7 +11525,7 @@
       <c r="A10" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="48"/>
+      <c r="B10" s="51"/>
       <c r="C10" s="10" t="s">
         <v>17</v>
       </c>
@@ -11529,7 +11541,7 @@
       <c r="A11" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="48"/>
+      <c r="B11" s="51"/>
       <c r="C11" s="10" t="s">
         <v>17</v>
       </c>
@@ -11545,7 +11557,7 @@
       <c r="A12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="48"/>
+      <c r="B12" s="51"/>
       <c r="C12" s="10" t="s">
         <v>17</v>
       </c>
@@ -11561,7 +11573,7 @@
       <c r="A13" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="48"/>
+      <c r="B13" s="51"/>
       <c r="C13" s="10" t="s">
         <v>17</v>
       </c>
@@ -11577,7 +11589,7 @@
       <c r="A14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="48"/>
+      <c r="B14" s="51"/>
       <c r="C14" s="10" t="s">
         <v>17</v>
       </c>
@@ -11593,7 +11605,7 @@
       <c r="A15" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="51"/>
       <c r="C15" s="10" t="s">
         <v>17</v>
       </c>
@@ -11609,7 +11621,7 @@
       <c r="A16" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="48"/>
+      <c r="B16" s="51"/>
       <c r="C16" s="10" t="s">
         <v>17</v>
       </c>
@@ -11625,7 +11637,7 @@
       <c r="A17" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="48"/>
+      <c r="B17" s="51"/>
       <c r="C17" s="10" t="s">
         <v>17</v>
       </c>
@@ -11641,7 +11653,7 @@
       <c r="A18" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="48"/>
+      <c r="B18" s="51"/>
       <c r="C18" s="10" t="s">
         <v>49</v>
       </c>
@@ -11657,7 +11669,7 @@
       <c r="A19" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="48"/>
+      <c r="B19" s="51"/>
       <c r="C19" s="10" t="s">
         <v>49</v>
       </c>
@@ -11673,7 +11685,7 @@
       <c r="A20" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="48"/>
+      <c r="B20" s="51"/>
       <c r="C20" s="10" t="s">
         <v>49</v>
       </c>
@@ -11689,7 +11701,7 @@
       <c r="A21" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="48"/>
+      <c r="B21" s="51"/>
       <c r="C21" s="10" t="s">
         <v>58</v>
       </c>
@@ -11705,7 +11717,7 @@
       <c r="A22" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="48"/>
+      <c r="B22" s="51"/>
       <c r="C22" s="10" t="s">
         <v>58</v>
       </c>
@@ -11721,7 +11733,7 @@
       <c r="A23" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="48"/>
+      <c r="B23" s="51"/>
       <c r="C23" s="10" t="s">
         <v>58</v>
       </c>
@@ -11737,7 +11749,7 @@
       <c r="A24" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="48"/>
+      <c r="B24" s="51"/>
       <c r="C24" s="10" t="s">
         <v>58</v>
       </c>
@@ -11753,7 +11765,7 @@
       <c r="A25" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="B25" s="48"/>
+      <c r="B25" s="51"/>
       <c r="C25" s="10" t="s">
         <v>58</v>
       </c>
@@ -11769,7 +11781,7 @@
       <c r="A26" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B26" s="48"/>
+      <c r="B26" s="51"/>
       <c r="C26" s="10" t="s">
         <v>58</v>
       </c>
@@ -11785,7 +11797,7 @@
       <c r="A27" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="B27" s="47" t="s">
+      <c r="B27" s="50" t="s">
         <v>77</v>
       </c>
       <c r="C27" s="15" t="s">
@@ -11807,7 +11819,7 @@
       <c r="A28" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="51"/>
       <c r="C28" s="15" t="s">
         <v>82</v>
       </c>
@@ -11828,7 +11840,7 @@
       <c r="A29" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B29" s="48"/>
+      <c r="B29" s="51"/>
       <c r="C29" s="15" t="s">
         <v>82</v>
       </c>
@@ -11849,7 +11861,7 @@
       <c r="A30" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B30" s="48"/>
+      <c r="B30" s="51"/>
       <c r="C30" s="15" t="s">
         <v>82</v>
       </c>
@@ -11870,7 +11882,7 @@
       <c r="A31" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="B31" s="48"/>
+      <c r="B31" s="51"/>
       <c r="C31" s="15" t="s">
         <v>82</v>
       </c>
@@ -11891,7 +11903,7 @@
       <c r="A32" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="48"/>
+      <c r="B32" s="51"/>
       <c r="C32" s="10" t="s">
         <v>87</v>
       </c>
@@ -11914,7 +11926,7 @@
       <c r="A33" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B33" s="48"/>
+      <c r="B33" s="51"/>
       <c r="C33" s="10" t="s">
         <v>87</v>
       </c>
@@ -11935,7 +11947,7 @@
       <c r="A34" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B34" s="48"/>
+      <c r="B34" s="51"/>
       <c r="C34" s="10" t="s">
         <v>87</v>
       </c>
@@ -11958,7 +11970,7 @@
       <c r="A35" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="B35" s="48"/>
+      <c r="B35" s="51"/>
       <c r="C35" s="10" t="s">
         <v>87</v>
       </c>
@@ -11981,7 +11993,7 @@
       <c r="A36" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="B36" s="48"/>
+      <c r="B36" s="51"/>
       <c r="C36" s="10" t="s">
         <v>87</v>
       </c>
@@ -12004,7 +12016,7 @@
       <c r="A37" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B37" s="48"/>
+      <c r="B37" s="51"/>
       <c r="C37" s="10" t="s">
         <v>98</v>
       </c>
@@ -12025,7 +12037,7 @@
       <c r="A38" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="48"/>
+      <c r="B38" s="51"/>
       <c r="C38" s="10" t="s">
         <v>98</v>
       </c>
@@ -12046,7 +12058,7 @@
       <c r="A39" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B39" s="48"/>
+      <c r="B39" s="51"/>
       <c r="C39" s="10" t="s">
         <v>98</v>
       </c>
@@ -12067,7 +12079,7 @@
       <c r="A40" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="B40" s="48"/>
+      <c r="B40" s="51"/>
       <c r="C40" s="10" t="s">
         <v>98</v>
       </c>
@@ -12088,7 +12100,7 @@
       <c r="A41" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="B41" s="48"/>
+      <c r="B41" s="51"/>
       <c r="C41" s="10" t="s">
         <v>98</v>
       </c>
@@ -12109,7 +12121,7 @@
       <c r="A42" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="B42" s="48"/>
+      <c r="B42" s="51"/>
       <c r="C42" s="10" t="s">
         <v>98</v>
       </c>
@@ -12130,7 +12142,7 @@
       <c r="A43" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="B43" s="48"/>
+      <c r="B43" s="51"/>
       <c r="C43" s="10" t="s">
         <v>98</v>
       </c>
@@ -12151,7 +12163,7 @@
       <c r="A44" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B44" s="48"/>
+      <c r="B44" s="51"/>
       <c r="C44" s="10" t="s">
         <v>98</v>
       </c>
@@ -12172,7 +12184,7 @@
       <c r="A45" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="B45" s="48"/>
+      <c r="B45" s="51"/>
       <c r="C45" s="10" t="s">
         <v>121</v>
       </c>
@@ -12193,7 +12205,7 @@
       <c r="A46" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B46" s="48"/>
+      <c r="B46" s="51"/>
       <c r="C46" s="10" t="s">
         <v>121</v>
       </c>
@@ -12214,7 +12226,7 @@
       <c r="A47" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B47" s="48"/>
+      <c r="B47" s="51"/>
       <c r="C47" s="10" t="s">
         <v>121</v>
       </c>
@@ -12235,7 +12247,7 @@
       <c r="A48" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B48" s="48"/>
+      <c r="B48" s="51"/>
       <c r="C48" s="10" t="s">
         <v>128</v>
       </c>
@@ -12256,7 +12268,7 @@
       <c r="A49" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="B49" s="48"/>
+      <c r="B49" s="51"/>
       <c r="C49" s="10" t="s">
         <v>128</v>
       </c>
@@ -12277,7 +12289,7 @@
       <c r="A50" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="B50" s="48"/>
+      <c r="B50" s="51"/>
       <c r="C50" s="10" t="s">
         <v>128</v>
       </c>
@@ -12298,7 +12310,7 @@
       <c r="A51" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B51" s="48"/>
+      <c r="B51" s="51"/>
       <c r="C51" s="10" t="s">
         <v>128</v>
       </c>
@@ -12319,7 +12331,7 @@
       <c r="A52" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="B52" s="48"/>
+      <c r="B52" s="51"/>
       <c r="C52" s="15" t="s">
         <v>139</v>
       </c>
@@ -12340,7 +12352,7 @@
       <c r="A53" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="B53" s="48"/>
+      <c r="B53" s="51"/>
       <c r="C53" s="15" t="s">
         <v>139</v>
       </c>
@@ -12361,7 +12373,7 @@
       <c r="A54" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="B54" s="48"/>
+      <c r="B54" s="51"/>
       <c r="C54" s="15" t="s">
         <v>139</v>
       </c>
@@ -12446,10 +12458,10 @@
       <c r="AB1" s="41"/>
     </row>
     <row r="2" spans="1:28" ht="63.75" customHeight="1">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="54" t="s">
         <v>170</v>
       </c>
       <c r="C2" s="20" t="s">
@@ -12488,8 +12500,8 @@
       <c r="AB2" s="20"/>
     </row>
     <row r="3" spans="1:28" ht="46.5" customHeight="1">
-      <c r="A3" s="49"/>
-      <c r="B3" s="51"/>
+      <c r="A3" s="52"/>
+      <c r="B3" s="54"/>
       <c r="C3" s="20" t="s">
         <v>172</v>
       </c>
@@ -12526,8 +12538,8 @@
       <c r="AB3" s="20"/>
     </row>
     <row r="4" spans="1:28" ht="22.5" customHeight="1">
-      <c r="A4" s="49"/>
-      <c r="B4" s="51"/>
+      <c r="A4" s="52"/>
+      <c r="B4" s="54"/>
       <c r="C4" s="20" t="s">
         <v>176</v>
       </c>
@@ -12562,8 +12574,8 @@
       <c r="AB4" s="20"/>
     </row>
     <row r="5" spans="1:28" ht="124.5" customHeight="1">
-      <c r="A5" s="49"/>
-      <c r="B5" s="51" t="s">
+      <c r="A5" s="52"/>
+      <c r="B5" s="54" t="s">
         <v>287</v>
       </c>
       <c r="C5" s="23" t="s">
@@ -12600,8 +12612,8 @@
       <c r="AB5" s="20"/>
     </row>
     <row r="6" spans="1:28" ht="28.5" customHeight="1">
-      <c r="A6" s="49"/>
-      <c r="B6" s="51"/>
+      <c r="A6" s="52"/>
+      <c r="B6" s="54"/>
       <c r="C6" s="20" t="s">
         <v>181</v>
       </c>
@@ -12636,8 +12648,8 @@
       <c r="AB6" s="20"/>
     </row>
     <row r="7" spans="1:28" ht="24.75" customHeight="1">
-      <c r="A7" s="49"/>
-      <c r="B7" s="51"/>
+      <c r="A7" s="52"/>
+      <c r="B7" s="54"/>
       <c r="C7" s="20" t="s">
         <v>184</v>
       </c>
@@ -12672,8 +12684,8 @@
       <c r="AB7" s="20"/>
     </row>
     <row r="8" spans="1:28" ht="23.25" customHeight="1">
-      <c r="A8" s="49"/>
-      <c r="B8" s="51"/>
+      <c r="A8" s="52"/>
+      <c r="B8" s="54"/>
       <c r="C8" s="20" t="s">
         <v>185</v>
       </c>
@@ -12708,8 +12720,8 @@
       <c r="AB8" s="20"/>
     </row>
     <row r="9" spans="1:28" ht="24.75" customHeight="1">
-      <c r="A9" s="49"/>
-      <c r="B9" s="51"/>
+      <c r="A9" s="52"/>
+      <c r="B9" s="54"/>
       <c r="C9" s="20" t="s">
         <v>188</v>
       </c>
@@ -12744,8 +12756,8 @@
       <c r="AB9" s="20"/>
     </row>
     <row r="10" spans="1:28" ht="26.25" customHeight="1">
-      <c r="A10" s="49"/>
-      <c r="B10" s="51"/>
+      <c r="A10" s="52"/>
+      <c r="B10" s="54"/>
       <c r="C10" s="20" t="s">
         <v>191</v>
       </c>
@@ -12782,8 +12794,8 @@
       <c r="AB10" s="20"/>
     </row>
     <row r="11" spans="1:28" ht="27.75" customHeight="1">
-      <c r="A11" s="49"/>
-      <c r="B11" s="51"/>
+      <c r="A11" s="52"/>
+      <c r="B11" s="54"/>
       <c r="C11" s="20" t="s">
         <v>195</v>
       </c>
@@ -12818,8 +12830,8 @@
       <c r="AB11" s="20"/>
     </row>
     <row r="12" spans="1:28" ht="24.75" customHeight="1">
-      <c r="A12" s="49"/>
-      <c r="B12" s="51"/>
+      <c r="A12" s="52"/>
+      <c r="B12" s="54"/>
       <c r="C12" s="20" t="s">
         <v>198</v>
       </c>
@@ -12854,8 +12866,8 @@
       <c r="AB12" s="20"/>
     </row>
     <row r="13" spans="1:28" ht="51.75" customHeight="1">
-      <c r="A13" s="49"/>
-      <c r="B13" s="51"/>
+      <c r="A13" s="52"/>
+      <c r="B13" s="54"/>
       <c r="C13" s="23" t="s">
         <v>201</v>
       </c>
@@ -12890,8 +12902,8 @@
       <c r="AB13" s="20"/>
     </row>
     <row r="14" spans="1:28" ht="33.75" customHeight="1">
-      <c r="A14" s="49"/>
-      <c r="B14" s="51"/>
+      <c r="A14" s="52"/>
+      <c r="B14" s="54"/>
       <c r="C14" s="20" t="s">
         <v>204</v>
       </c>
@@ -12928,8 +12940,8 @@
       <c r="AB14" s="20"/>
     </row>
     <row r="15" spans="1:28" s="25" customFormat="1" ht="30.75" customHeight="1">
-      <c r="A15" s="49"/>
-      <c r="B15" s="51" t="s">
+      <c r="A15" s="52"/>
+      <c r="B15" s="54" t="s">
         <v>206</v>
       </c>
       <c r="C15" s="24" t="s">
@@ -12966,8 +12978,8 @@
       <c r="AB15" s="24"/>
     </row>
     <row r="16" spans="1:28" s="25" customFormat="1" ht="27" customHeight="1">
-      <c r="A16" s="49"/>
-      <c r="B16" s="51"/>
+      <c r="A16" s="52"/>
+      <c r="B16" s="54"/>
       <c r="C16" s="24" t="s">
         <v>210</v>
       </c>
@@ -13002,8 +13014,8 @@
       <c r="AB16" s="24"/>
     </row>
     <row r="17" spans="1:28" s="25" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A17" s="49"/>
-      <c r="B17" s="51"/>
+      <c r="A17" s="52"/>
+      <c r="B17" s="54"/>
       <c r="C17" s="24" t="s">
         <v>212</v>
       </c>
@@ -13038,8 +13050,8 @@
       <c r="AB17" s="24"/>
     </row>
     <row r="18" spans="1:28" s="25" customFormat="1" ht="26.25" customHeight="1">
-      <c r="A18" s="49"/>
-      <c r="B18" s="51"/>
+      <c r="A18" s="52"/>
+      <c r="B18" s="54"/>
       <c r="C18" s="24" t="s">
         <v>215</v>
       </c>
@@ -13074,8 +13086,8 @@
       <c r="AB18" s="24"/>
     </row>
     <row r="19" spans="1:28" s="25" customFormat="1" ht="32.25" customHeight="1">
-      <c r="A19" s="49"/>
-      <c r="B19" s="51"/>
+      <c r="A19" s="52"/>
+      <c r="B19" s="54"/>
       <c r="C19" s="24" t="s">
         <v>218</v>
       </c>
@@ -13110,8 +13122,8 @@
       <c r="AB19" s="24"/>
     </row>
     <row r="20" spans="1:28" s="25" customFormat="1" ht="45.75" customHeight="1">
-      <c r="A20" s="49"/>
-      <c r="B20" s="51"/>
+      <c r="A20" s="52"/>
+      <c r="B20" s="54"/>
       <c r="C20" s="23" t="s">
         <v>221</v>
       </c>
@@ -13146,8 +13158,8 @@
       <c r="AB20" s="24"/>
     </row>
     <row r="21" spans="1:28" ht="33.75" customHeight="1">
-      <c r="A21" s="49"/>
-      <c r="B21" s="51" t="s">
+      <c r="A21" s="52"/>
+      <c r="B21" s="54" t="s">
         <v>224</v>
       </c>
       <c r="C21" s="20" t="s">
@@ -13184,8 +13196,8 @@
       <c r="AB21" s="20"/>
     </row>
     <row r="22" spans="1:28" ht="27" customHeight="1">
-      <c r="A22" s="49"/>
-      <c r="B22" s="51"/>
+      <c r="A22" s="52"/>
+      <c r="B22" s="54"/>
       <c r="C22" s="20" t="s">
         <v>228</v>
       </c>
@@ -13220,8 +13232,8 @@
       <c r="AB22" s="20"/>
     </row>
     <row r="23" spans="1:28" ht="28.5" customHeight="1">
-      <c r="A23" s="49"/>
-      <c r="B23" s="51"/>
+      <c r="A23" s="52"/>
+      <c r="B23" s="54"/>
       <c r="C23" s="20" t="s">
         <v>231</v>
       </c>
@@ -13256,8 +13268,8 @@
       <c r="AB23" s="20"/>
     </row>
     <row r="24" spans="1:28" ht="28.5" customHeight="1">
-      <c r="A24" s="49"/>
-      <c r="B24" s="51"/>
+      <c r="A24" s="52"/>
+      <c r="B24" s="54"/>
       <c r="C24" s="20" t="s">
         <v>234</v>
       </c>
@@ -13292,8 +13304,8 @@
       <c r="AB24" s="20"/>
     </row>
     <row r="25" spans="1:28" ht="27.75" customHeight="1">
-      <c r="A25" s="49"/>
-      <c r="B25" s="51"/>
+      <c r="A25" s="52"/>
+      <c r="B25" s="54"/>
       <c r="C25" s="20" t="s">
         <v>236</v>
       </c>
@@ -13328,8 +13340,8 @@
       <c r="AB25" s="20"/>
     </row>
     <row r="26" spans="1:28" ht="25.5" customHeight="1">
-      <c r="A26" s="49"/>
-      <c r="B26" s="51"/>
+      <c r="A26" s="52"/>
+      <c r="B26" s="54"/>
       <c r="C26" s="20" t="s">
         <v>237</v>
       </c>
@@ -13364,8 +13376,8 @@
       <c r="AB26" s="20"/>
     </row>
     <row r="27" spans="1:28" ht="27" customHeight="1">
-      <c r="A27" s="49"/>
-      <c r="B27" s="51"/>
+      <c r="A27" s="52"/>
+      <c r="B27" s="54"/>
       <c r="C27" s="20" t="s">
         <v>240</v>
       </c>
@@ -13400,8 +13412,8 @@
       <c r="AB27" s="20"/>
     </row>
     <row r="28" spans="1:28" ht="58.5" customHeight="1">
-      <c r="A28" s="49"/>
-      <c r="B28" s="51"/>
+      <c r="A28" s="52"/>
+      <c r="B28" s="54"/>
       <c r="C28" s="20" t="s">
         <v>243</v>
       </c>
@@ -13437,123 +13449,123 @@
       <c r="AA28" s="20"/>
       <c r="AB28" s="20"/>
     </row>
-    <row r="29" spans="1:28" s="54" customFormat="1" ht="44.25" customHeight="1">
-      <c r="A29" s="49"/>
-      <c r="B29" s="52" t="s">
+    <row r="29" spans="1:28" s="48" customFormat="1" ht="44.25" customHeight="1">
+      <c r="A29" s="52"/>
+      <c r="B29" s="55" t="s">
         <v>247</v>
       </c>
-      <c r="C29" s="53" t="s">
+      <c r="C29" s="47" t="s">
         <v>250</v>
       </c>
-      <c r="D29" s="53" t="s">
+      <c r="D29" s="47" t="s">
         <v>249</v>
       </c>
-      <c r="E29" s="53" t="s">
+      <c r="E29" s="47" t="s">
         <v>284</v>
       </c>
-      <c r="F29" s="53" t="s">
+      <c r="F29" s="47" t="s">
         <v>292</v>
       </c>
-      <c r="G29" s="53"/>
-      <c r="H29" s="53"/>
-      <c r="I29" s="53"/>
-      <c r="J29" s="53"/>
-      <c r="K29" s="53"/>
-      <c r="L29" s="53"/>
-      <c r="M29" s="53"/>
-      <c r="N29" s="53"/>
-      <c r="O29" s="53"/>
-      <c r="P29" s="53"/>
-      <c r="Q29" s="53"/>
-      <c r="R29" s="53"/>
-      <c r="S29" s="53"/>
-      <c r="T29" s="53"/>
-      <c r="U29" s="53"/>
-      <c r="V29" s="53"/>
-      <c r="W29" s="53"/>
-      <c r="X29" s="53"/>
-      <c r="Y29" s="53"/>
-      <c r="Z29" s="53"/>
-      <c r="AA29" s="53"/>
-      <c r="AB29" s="53"/>
-    </row>
-    <row r="30" spans="1:28" ht="36" customHeight="1">
-      <c r="A30" s="49"/>
-      <c r="B30" s="52"/>
-      <c r="C30" s="20" t="s">
+      <c r="G29" s="47"/>
+      <c r="H29" s="47"/>
+      <c r="I29" s="47"/>
+      <c r="J29" s="47"/>
+      <c r="K29" s="47"/>
+      <c r="L29" s="47"/>
+      <c r="M29" s="47"/>
+      <c r="N29" s="47"/>
+      <c r="O29" s="47"/>
+      <c r="P29" s="47"/>
+      <c r="Q29" s="47"/>
+      <c r="R29" s="47"/>
+      <c r="S29" s="47"/>
+      <c r="T29" s="47"/>
+      <c r="U29" s="47"/>
+      <c r="V29" s="47"/>
+      <c r="W29" s="47"/>
+      <c r="X29" s="47"/>
+      <c r="Y29" s="47"/>
+      <c r="Z29" s="47"/>
+      <c r="AA29" s="47"/>
+      <c r="AB29" s="47"/>
+    </row>
+    <row r="30" spans="1:28" s="57" customFormat="1" ht="36" customHeight="1">
+      <c r="A30" s="52"/>
+      <c r="B30" s="55"/>
+      <c r="C30" s="56" t="s">
         <v>251</v>
       </c>
-      <c r="D30" s="20" t="s">
+      <c r="D30" s="56" t="s">
         <v>248</v>
       </c>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="56" t="s">
         <v>285</v>
       </c>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
-      <c r="L30" s="20"/>
-      <c r="M30" s="20"/>
-      <c r="N30" s="20"/>
-      <c r="O30" s="20"/>
-      <c r="P30" s="20"/>
-      <c r="Q30" s="20"/>
-      <c r="R30" s="20"/>
-      <c r="S30" s="20"/>
-      <c r="T30" s="20"/>
-      <c r="U30" s="20"/>
-      <c r="V30" s="20"/>
-      <c r="W30" s="20"/>
-      <c r="X30" s="20"/>
-      <c r="Y30" s="20"/>
-      <c r="Z30" s="20"/>
-      <c r="AA30" s="20"/>
-      <c r="AB30" s="20"/>
-    </row>
-    <row r="31" spans="1:28" s="54" customFormat="1">
-      <c r="A31" s="49"/>
-      <c r="B31" s="52"/>
-      <c r="C31" s="53" t="s">
+      <c r="F30" s="56"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="56"/>
+      <c r="I30" s="56"/>
+      <c r="J30" s="56"/>
+      <c r="K30" s="56"/>
+      <c r="L30" s="56"/>
+      <c r="M30" s="56"/>
+      <c r="N30" s="56"/>
+      <c r="O30" s="56"/>
+      <c r="P30" s="56"/>
+      <c r="Q30" s="56"/>
+      <c r="R30" s="56"/>
+      <c r="S30" s="56"/>
+      <c r="T30" s="56"/>
+      <c r="U30" s="56"/>
+      <c r="V30" s="56"/>
+      <c r="W30" s="56"/>
+      <c r="X30" s="56"/>
+      <c r="Y30" s="56"/>
+      <c r="Z30" s="56"/>
+      <c r="AA30" s="56"/>
+      <c r="AB30" s="56"/>
+    </row>
+    <row r="31" spans="1:28" s="48" customFormat="1">
+      <c r="A31" s="52"/>
+      <c r="B31" s="55"/>
+      <c r="C31" s="47" t="s">
         <v>252</v>
       </c>
-      <c r="D31" s="55" t="s">
+      <c r="D31" s="49" t="s">
         <v>253</v>
       </c>
-      <c r="E31" s="53" t="s">
+      <c r="E31" s="47" t="s">
         <v>254</v>
       </c>
-      <c r="F31" s="53"/>
-      <c r="G31" s="53"/>
-      <c r="H31" s="53"/>
-      <c r="I31" s="53"/>
-      <c r="J31" s="53"/>
-      <c r="K31" s="53"/>
-      <c r="L31" s="53"/>
-      <c r="M31" s="53"/>
-      <c r="N31" s="53"/>
-      <c r="O31" s="53"/>
-      <c r="P31" s="53"/>
-      <c r="Q31" s="53"/>
-      <c r="R31" s="53"/>
-      <c r="S31" s="53"/>
-      <c r="T31" s="53"/>
-      <c r="U31" s="53"/>
-      <c r="V31" s="53"/>
-      <c r="W31" s="53"/>
-      <c r="X31" s="53"/>
-      <c r="Y31" s="53"/>
-      <c r="Z31" s="53"/>
-      <c r="AA31" s="53"/>
-      <c r="AB31" s="53"/>
+      <c r="F31" s="47"/>
+      <c r="G31" s="47"/>
+      <c r="H31" s="47"/>
+      <c r="I31" s="47"/>
+      <c r="J31" s="47"/>
+      <c r="K31" s="47"/>
+      <c r="L31" s="47"/>
+      <c r="M31" s="47"/>
+      <c r="N31" s="47"/>
+      <c r="O31" s="47"/>
+      <c r="P31" s="47"/>
+      <c r="Q31" s="47"/>
+      <c r="R31" s="47"/>
+      <c r="S31" s="47"/>
+      <c r="T31" s="47"/>
+      <c r="U31" s="47"/>
+      <c r="V31" s="47"/>
+      <c r="W31" s="47"/>
+      <c r="X31" s="47"/>
+      <c r="Y31" s="47"/>
+      <c r="Z31" s="47"/>
+      <c r="AA31" s="47"/>
+      <c r="AB31" s="47"/>
     </row>
     <row r="32" spans="1:28" ht="51">
-      <c r="A32" s="50" t="s">
+      <c r="A32" s="53" t="s">
         <v>255</v>
       </c>
-      <c r="B32" s="49" t="s">
+      <c r="B32" s="52" t="s">
         <v>267</v>
       </c>
       <c r="C32" s="20" t="s">
@@ -13592,8 +13604,8 @@
       <c r="AB32" s="20"/>
     </row>
     <row r="33" spans="1:28" ht="25.5">
-      <c r="A33" s="50"/>
-      <c r="B33" s="49"/>
+      <c r="A33" s="53"/>
+      <c r="B33" s="52"/>
       <c r="C33" s="20" t="s">
         <v>268</v>
       </c>
@@ -13628,8 +13640,8 @@
       <c r="AB33" s="20"/>
     </row>
     <row r="34" spans="1:28" ht="25.5">
-      <c r="A34" s="50"/>
-      <c r="B34" s="49"/>
+      <c r="A34" s="53"/>
+      <c r="B34" s="52"/>
       <c r="C34" s="20" t="s">
         <v>265</v>
       </c>
@@ -13666,8 +13678,8 @@
       <c r="AB34" s="20"/>
     </row>
     <row r="35" spans="1:28" ht="56.25" customHeight="1">
-      <c r="A35" s="50"/>
-      <c r="B35" s="49"/>
+      <c r="A35" s="53"/>
+      <c r="B35" s="52"/>
       <c r="C35" s="20" t="s">
         <v>83</v>
       </c>
@@ -13704,8 +13716,8 @@
       <c r="AB35" s="20"/>
     </row>
     <row r="36" spans="1:28" s="29" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A36" s="50"/>
-      <c r="B36" s="49"/>
+      <c r="A36" s="53"/>
+      <c r="B36" s="52"/>
       <c r="C36" s="23" t="s">
         <v>84</v>
       </c>
@@ -13725,8 +13737,8 @@
       <c r="K36" s="28"/>
     </row>
     <row r="37" spans="1:28" s="29" customFormat="1" ht="45" customHeight="1">
-      <c r="A37" s="50"/>
-      <c r="B37" s="49"/>
+      <c r="A37" s="53"/>
+      <c r="B37" s="52"/>
       <c r="C37" s="34" t="s">
         <v>269</v>
       </c>

</xml_diff>